<commit_message>
Update to Choropleth File
New India-Choropleth-V2 created to load files from GitHub
</commit_message>
<xml_diff>
--- a/Capex/election_data/Assembly-elections.xlsx
+++ b/Capex/election_data/Assembly-elections.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iimv1-my.sharepoint.com/personal/kalyan_iimv_ac_in/Documents/Python-Exercise-KK/Kalyan-Jupyter-Notebooks/Capex/election_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e46a4301436fbcaf/Kalyan/KK-Python/Kalyan-Jupyter-Notebooks/Capex/election_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{7BCBB9CB-93D5-6845-8A89-831BE904A6DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D85AC640-633A-DD4E-A8EC-86A69B15D51D}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{7BCBB9CB-93D5-6845-8A89-831BE904A6DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76D4CC2B-324F-9247-BBEF-788E8237E94E}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="980" windowWidth="27240" windowHeight="14600" firstSheet="1" activeTab="1" xr2:uid="{F4A064C8-720D-0840-BC92-FFF0422F84E6}"/>
+    <workbookView xWindow="780" yWindow="980" windowWidth="27240" windowHeight="14600" xr2:uid="{F4A064C8-720D-0840-BC92-FFF0422F84E6}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="AC poll years" sheetId="1" r:id="rId1"/>
+    <sheet name="AC Election Years" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="281">
   <si>
     <t>STATES</t>
   </si>
@@ -878,6 +878,9 @@
   </si>
   <si>
     <t> 1971  </t>
+  </si>
+  <si>
+    <t>State Formation Year</t>
   </si>
 </sst>
 </file>
@@ -913,8 +916,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -933,9 +939,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -973,7 +979,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1079,7 +1085,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1221,7 +1227,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1243,6 +1249,7 @@
     <col min="15" max="15" width="7.5" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
@@ -1252,6 +1259,9 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="R1" t="s">
+        <v>280</v>
+      </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -1304,6 +1314,9 @@
       </c>
       <c r="Q2" t="s">
         <v>18</v>
+      </c>
+      <c r="R2">
+        <v>1950</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
@@ -2597,1322 +2610,1324 @@
   <dimension ref="A1:AF19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11" style="1"/>
+    <col min="2" max="2" width="14" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="O2" t="s">
+      <c r="O2" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="Q2" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="S2">
+      <c r="S2" s="1">
         <v>2023</v>
       </c>
-      <c r="T2" t="s">
+      <c r="T2" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="U2" t="s">
+      <c r="U2" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="V2" t="s">
+      <c r="V2" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="X2" t="s">
+      <c r="X2" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Y2" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="Z2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AA2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AB2">
+      <c r="AB2" s="1">
         <v>2018</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AC2" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AD2" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AE2" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AF2" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="N3" t="s">
+      <c r="N3" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="O3" t="s">
+      <c r="O3" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="P3" t="s">
+      <c r="P3" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="Q3" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="S3" t="s">
+      <c r="S3" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="T3" t="s">
+      <c r="T3" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="U3" t="s">
+      <c r="U3" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="V3" t="s">
+      <c r="V3" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="W3" t="s">
+      <c r="W3" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="X3" t="s">
+      <c r="X3" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Y3" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="Z3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AA3" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AC3" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AD3" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="AE3" t="s">
+      <c r="AE3" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="AF3" t="s">
+      <c r="AF3" s="1" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N4" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O4" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P4" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="R4" t="s">
+      <c r="R4" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="S4" t="s">
+      <c r="S4" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="T4" t="s">
+      <c r="T4" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="U4" t="s">
+      <c r="U4" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="V4" t="s">
+      <c r="V4" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="W4" t="s">
+      <c r="W4" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="X4" t="s">
+      <c r="X4" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="Y4" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="Z4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AA4" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="AC4" t="s">
+      <c r="AC4" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="AD4" t="s">
+      <c r="AD4" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="AE4" t="s">
+      <c r="AE4" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="AF4" t="s">
+      <c r="AF4" s="1" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L5" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M5" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="N5" t="s">
+      <c r="N5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="O5" t="s">
+      <c r="O5" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="P5" t="s">
+      <c r="P5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="Q5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="R5" t="s">
+      <c r="R5" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="S5" t="s">
+      <c r="S5" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="T5" t="s">
+      <c r="T5" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="U5" t="s">
+      <c r="U5" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="V5" t="s">
+      <c r="V5" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="W5" t="s">
+      <c r="W5" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="X5" t="s">
+      <c r="X5" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="Y5" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="Z5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="AA5" t="s">
+      <c r="AA5" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AC5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="AD5" t="s">
+      <c r="AD5" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="AE5" t="s">
+      <c r="AE5" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="AF5" t="s">
+      <c r="AF5" s="1" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="L6" t="s">
+      <c r="L6" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="N6" t="s">
+      <c r="N6" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="O6" t="s">
+      <c r="O6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="P6" t="s">
+      <c r="P6" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="Q6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="R6" t="s">
+      <c r="R6" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="S6" t="s">
+      <c r="S6" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="T6" t="s">
+      <c r="T6" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="U6" t="s">
+      <c r="U6" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="V6" t="s">
+      <c r="V6" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="W6" t="s">
+      <c r="W6" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="X6" t="s">
+      <c r="X6" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="Y6" t="s">
+      <c r="Y6" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="Z6" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AA6" t="s">
+      <c r="AA6" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="AC6" t="s">
+      <c r="AC6" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="AD6" t="s">
+      <c r="AD6" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="AE6" t="s">
+      <c r="AE6" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="AF6" t="s">
+      <c r="AF6" s="1" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L7" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="N7" t="s">
+      <c r="N7" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="O7" t="s">
+      <c r="O7" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="P7" t="s">
+      <c r="P7" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="Q7" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="R7" t="s">
+      <c r="R7" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="S7" t="s">
+      <c r="S7" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="T7" t="s">
+      <c r="T7" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="U7" t="s">
+      <c r="U7" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="V7" t="s">
+      <c r="V7" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="W7" t="s">
+      <c r="W7" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="X7">
+      <c r="X7" s="1">
         <v>1996</v>
       </c>
-      <c r="Y7" t="s">
+      <c r="Y7" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="Z7" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="AA7" t="s">
+      <c r="AA7" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="AC7" t="s">
+      <c r="AC7" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="AD7" t="s">
+      <c r="AD7" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="AE7" t="s">
+      <c r="AE7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AF7" t="s">
+      <c r="AF7" s="1" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="L8" t="s">
+      <c r="L8" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N8" t="s">
+      <c r="N8" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="O8" t="s">
+      <c r="O8" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="P8" t="s">
+      <c r="P8" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="Q8" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="R8" t="s">
+      <c r="R8" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="S8" t="s">
+      <c r="S8" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="T8" t="s">
+      <c r="T8" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="U8" t="s">
+      <c r="U8" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="V8" t="s">
+      <c r="V8" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="W8" t="s">
+      <c r="W8" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="X8" t="s">
+      <c r="X8" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="Y8" t="s">
+      <c r="Y8" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="Z8" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="AA8" t="s">
+      <c r="AA8" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AC8" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="AD8" t="s">
+      <c r="AD8" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="AF8" t="s">
+      <c r="AF8" s="1" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="N9" t="s">
+      <c r="N9" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="O9" t="s">
+      <c r="O9" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="P9" t="s">
+      <c r="P9" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="Q9" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="R9" t="s">
+      <c r="R9" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="S9" t="s">
+      <c r="S9" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="T9" t="s">
+      <c r="T9" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="U9" t="s">
+      <c r="U9" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="V9" t="s">
+      <c r="V9" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="W9" t="s">
+      <c r="W9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="X9" t="s">
+      <c r="X9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="Y9" t="s">
+      <c r="Y9" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="Z9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="AA9" t="s">
+      <c r="AA9" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="AC9" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="AD9" t="s">
+      <c r="AD9" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="AF9" t="s">
+      <c r="AF9" s="1" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="N10" t="s">
+      <c r="N10" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="O10" t="s">
+      <c r="O10" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="P10" t="s">
+      <c r="P10" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="Q10" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="R10" t="s">
+      <c r="R10" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="S10" t="s">
+      <c r="S10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="T10" t="s">
+      <c r="T10" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="U10" t="s">
+      <c r="U10" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="V10" t="s">
+      <c r="V10" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="W10" t="s">
+      <c r="W10" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="X10" t="s">
+      <c r="X10" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="Y10" t="s">
+      <c r="Y10" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="Z10" t="s">
+      <c r="Z10" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="AA10" t="s">
+      <c r="AA10" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="AC10" t="s">
+      <c r="AC10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="AD10" t="s">
+      <c r="AD10" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="AF10" t="s">
+      <c r="AF10" s="1" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L11" t="s">
+      <c r="L11" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="N11" t="s">
+      <c r="N11" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="O11" t="s">
+      <c r="O11" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="P11" t="s">
+      <c r="P11" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="Q11" t="s">
+      <c r="Q11" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="R11" t="s">
+      <c r="R11" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="S11" t="s">
+      <c r="S11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="T11" t="s">
+      <c r="T11" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="U11" t="s">
+      <c r="U11" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="V11" t="s">
+      <c r="V11" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="W11" t="s">
+      <c r="W11" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="X11" t="s">
+      <c r="X11" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="Y11" t="s">
+      <c r="Y11" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="AA11" t="s">
+      <c r="AA11" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="AC11" t="s">
+      <c r="AC11" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="AD11" t="s">
+      <c r="AD11" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="AF11" t="s">
+      <c r="AF11" s="1" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="K12" t="s">
+      <c r="K12" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N12" t="s">
+      <c r="N12" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="O12" t="s">
+      <c r="O12" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="P12" t="s">
+      <c r="P12" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="Q12" t="s">
+      <c r="Q12" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="R12" t="s">
+      <c r="R12" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="S12" t="s">
+      <c r="S12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="T12" t="s">
+      <c r="T12" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="U12" t="s">
+      <c r="U12" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="V12" t="s">
+      <c r="V12" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="W12" t="s">
+      <c r="W12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="X12" t="s">
+      <c r="X12" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="Y12" t="s">
+      <c r="Y12" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="AA12" t="s">
+      <c r="AA12" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="AC12" t="s">
+      <c r="AC12" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AD12" t="s">
+      <c r="AD12" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="AF12" t="s">
+      <c r="AF12" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="K13" t="s">
+      <c r="K13" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="N13" t="s">
+      <c r="N13" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="O13" t="s">
+      <c r="O13" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="P13" t="s">
+      <c r="P13" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="Q13" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="R13" t="s">
+      <c r="R13" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="T13" t="s">
+      <c r="T13" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="U13" t="s">
+      <c r="U13" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="V13" t="s">
+      <c r="V13" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="W13" t="s">
+      <c r="W13" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="X13" t="s">
+      <c r="X13" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="Y13" t="s">
+      <c r="Y13" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="AA13" t="s">
+      <c r="AA13" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="AC13" t="s">
+      <c r="AC13" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="AD13" t="s">
+      <c r="AD13" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="AF13" t="s">
+      <c r="AF13" s="1" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K14" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="N14" t="s">
+      <c r="N14" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="O14" t="s">
+      <c r="O14" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="P14" t="s">
+      <c r="P14" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="Q14" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="R14" t="s">
+      <c r="R14" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="U14" t="s">
+      <c r="U14" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="V14" t="s">
+      <c r="V14" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="W14" t="s">
+      <c r="W14" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="X14" t="s">
+      <c r="X14" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="Y14" t="s">
+      <c r="Y14" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="AA14" t="s">
+      <c r="AA14" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AC14" t="s">
+      <c r="AC14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="AD14" t="s">
+      <c r="AD14" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="AF14" t="s">
+      <c r="AF14" s="1" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="K15" t="s">
+      <c r="K15" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="N15" t="s">
+      <c r="N15" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="O15" t="s">
+      <c r="O15" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="P15" t="s">
+      <c r="P15" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="U15" t="s">
+      <c r="U15" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="V15" t="s">
+      <c r="V15" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="W15" t="s">
+      <c r="W15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="X15" t="s">
+      <c r="X15" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="Y15" t="s">
+      <c r="Y15" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="AD15" t="s">
+      <c r="AD15" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="AF15" t="s">
+      <c r="AF15" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="N16" t="s">
+      <c r="N16" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="O16" t="s">
+      <c r="O16" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="P16" t="s">
+      <c r="P16" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="U16" t="s">
+      <c r="U16" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="V16" t="s">
+      <c r="V16" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="W16" t="s">
+      <c r="W16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="X16" t="s">
+      <c r="X16" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="Y16" t="s">
+      <c r="Y16" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="AD16" t="s">
+      <c r="AD16" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="AF16" t="s">
+      <c r="AF16" s="1" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="17" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="O17" t="s">
+      <c r="O17" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="V17" t="s">
+      <c r="V17" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="W17" t="s">
+      <c r="W17" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="AD17" t="s">
+      <c r="AD17" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="AF17" t="s">
+      <c r="AF17" s="1" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="18" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="E18" t="s">
+      <c r="E18" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AD18" t="s">
+      <c r="AD18" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="AF18" t="s">
+      <c r="AF18" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="19" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="AD19" t="s">
+      <c r="AD19" s="1" t="s">
         <v>115</v>
       </c>
     </row>

</xml_diff>